<commit_message>
Add overnight monster implementations and AI coverage
</commit_message>
<xml_diff>
--- a/docs/reference/srd_Creatures_Trimmed_V4.xlsx
+++ b/docs/reference/srd_Creatures_Trimmed_V4.xlsx
@@ -8887,7 +8887,7 @@
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -9063,7 +9063,7 @@
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -9943,7 +9943,7 @@
       </c>
       <c r="R110" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -10647,7 +10647,7 @@
       </c>
       <c r="R118" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -12495,7 +12495,7 @@
       </c>
       <c r="R139" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -12583,7 +12583,7 @@
       </c>
       <c r="R140" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -23763,32 +23763,19 @@
         </is>
       </c>
     </row>
-    <row r="268">
-    </row>
-    <row r="269">
-    </row>
-    <row r="270">
-    </row>
-    <row r="271">
-    </row>
-    <row r="272">
-    </row>
-    <row r="273">
-    </row>
-    <row r="274">
-    </row>
-    <row r="275">
-    </row>
-    <row r="276">
-    </row>
-    <row r="277">
-    </row>
-    <row r="278">
-    </row>
-    <row r="279">
-    </row>
-    <row r="280">
-    </row>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
+    <row r="275"/>
+    <row r="276"/>
+    <row r="277"/>
+    <row r="278"/>
+    <row r="279"/>
+    <row r="280"/>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Track non-SRD priority monsters
</commit_message>
<xml_diff>
--- a/docs/reference/srd_Creatures_Trimmed_V4.xlsx
+++ b/docs/reference/srd_Creatures_Trimmed_V4.xlsx
@@ -260,7 +260,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R287"/>
+  <dimension ref="A1:R290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24384,6 +24384,261 @@
         </is>
       </c>
     </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Bard</t>
+        </is>
+      </c>
+      <c r="B288" t="n">
+        <v>2</v>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Humanoid (Bard)</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Non-SRD Priority Targets</t>
+        </is>
+      </c>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G288" t="inlineStr">
+        <is>
+          <t>30 ft.</t>
+        </is>
+      </c>
+      <c r="H288" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>Yes - MotM/Volo-style magical NPC; confirm exact action model during implementation.</t>
+        </is>
+      </c>
+      <c r="P288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q288" t="inlineStr">
+        <is>
+          <t>https://www.aidedd.org/dnd/monstres.php?vo=bard</t>
+        </is>
+      </c>
+      <c r="R288" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Hobgoblin Devastator</t>
+        </is>
+      </c>
+      <c r="B289" t="n">
+        <v>4</v>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Fey (Goblinoid)</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>Non-SRD Priority Targets</t>
+        </is>
+      </c>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G289" t="inlineStr">
+        <is>
+          <t>30 ft.</t>
+        </is>
+      </c>
+      <c r="H289" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="N289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>Yes - Uses magical ranged offense and spellcasting; confirm exact action model during implementation.</t>
+        </is>
+      </c>
+      <c r="P289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q289" t="inlineStr">
+        <is>
+          <t>https://www.aidedd.org/dnd/monstres.php?vo=hobgoblin-devastator</t>
+        </is>
+      </c>
+      <c r="R289" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Flameskull</t>
+        </is>
+      </c>
+      <c r="B290" t="n">
+        <v>4</v>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Undead</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>Non-SRD Priority Targets</t>
+        </is>
+      </c>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>Tiny</t>
+        </is>
+      </c>
+      <c r="G290" t="inlineStr">
+        <is>
+          <t>0 ft., Fly 40 ft. (hover)</t>
+        </is>
+      </c>
+      <c r="H290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="K290" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="M290" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="N290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>Yes - The flameskull uses Fire Ray twice.</t>
+        </is>
+      </c>
+      <c r="P290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="Q290" t="inlineStr">
+        <is>
+          <t>https://www.aidedd.org/dnd/monstres.php?vo=flameskull</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>